<commit_message>
updated the empty experiment (blank miappe) with LOTS of help to fill it properly
</commit_message>
<xml_diff>
--- a/exp_database/empty_experiment/output/miappe_template_filled.xlsx
+++ b/exp_database/empty_experiment/output/miappe_template_filled.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="464">
   <si>
     <t xml:space="preserve">README</t>
   </si>
@@ -1381,7 +1381,13 @@
     <t xml:space="preserve">OpenSilex Version</t>
   </si>
   <si>
-    <t xml:space="preserve">can be prefilled</t>
+    <t xml:space="preserve">start_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">end_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rdf_type</t>
   </si>
   <si>
     <t xml:space="preserve">Accession number</t>
@@ -1397,6 +1403,21 @@
   </si>
   <si>
     <t xml:space="preserve">expeFactorValuesDesc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabular Data Provenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datafiles1 Provenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datafile1_rdf_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datafiles2 Provenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datafile2_rdf_type</t>
   </si>
   <si>
     <t xml:space="preserve">variableURI</t>
@@ -1594,18 +1615,12 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC9DAF8"/>
-        <bgColor rgb="FFC0C0C0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -1668,191 +1683,191 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1865,66 +1880,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFC9DAF8"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -7033,10 +6988,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
     </row>
     <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -7096,8 +7051,12 @@
       <c r="G1" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="17"/>
-      <c r="I1" s="18"/>
+      <c r="H1" s="17" t="s">
+        <v>446</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>447</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -9202,16 +9161,17 @@
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="14.43359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="23.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="8" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="7" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9221,17 +9181,16 @@
       <c r="B1" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="18" t="s">
+      <c r="C1" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>137</v>
       </c>
+      <c r="E1" s="17" t="s">
+        <v>138</v>
+      </c>
       <c r="F1" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="G1" s="17" t="s">
         <v>139</v>
       </c>
     </row>
@@ -10251,7 +10210,7 @@
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q1048576"/>
+  <dimension ref="A1:P1048576"/>
   <sheetFormatPr defaultColWidth="14.43359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.57"/>
@@ -10262,14 +10221,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="23.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="16.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10280,46 +10239,43 @@
       <c r="C1" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="D1" s="39" t="s">
-        <v>446</v>
-      </c>
-      <c r="E1" s="40" t="s">
+      <c r="D1" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="E1" s="39" t="s">
         <v>197</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>198</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>199</v>
       </c>
-      <c r="H1" s="40" t="s">
+      <c r="H1" s="39" t="s">
         <v>200</v>
       </c>
       <c r="I1" s="39" t="s">
-        <v>446</v>
-      </c>
-      <c r="J1" s="40" t="s">
         <v>201</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="J1" s="39" t="s">
         <v>207</v>
       </c>
-      <c r="L1" s="40" t="s">
+      <c r="K1" s="39" t="s">
         <v>208</v>
       </c>
-      <c r="M1" s="40" t="s">
-        <v>447</v>
-      </c>
-      <c r="N1" s="40" t="s">
-        <v>448</v>
-      </c>
-      <c r="O1" s="40" t="s">
+      <c r="L1" s="39" t="s">
+        <v>449</v>
+      </c>
+      <c r="M1" s="39" t="s">
+        <v>450</v>
+      </c>
+      <c r="N1" s="39" t="s">
         <v>265</v>
       </c>
-      <c r="P1" s="40" t="s">
-        <v>449</v>
-      </c>
-      <c r="Q1" s="41"/>
+      <c r="O1" s="39" t="s">
+        <v>451</v>
+      </c>
+      <c r="P1" s="40"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -11338,31 +11294,40 @@
   </sheetPr>
   <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="21.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.44"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="H1" s="0" t="s">
-        <v>450</v>
+      <c r="H1" s="1" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="1048527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -11457,29 +11422,29 @@
         <v>285</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>451</v>
-      </c>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="43"/>
-      <c r="Z1" s="43"/>
+        <v>453</v>
+      </c>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="42"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="42"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -12503,7 +12468,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="20.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="5" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="10" style="1" width="14.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12519,26 +12489,36 @@
       <c r="D1" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
-      <c r="X1" s="43"/>
+      <c r="E1" s="17" t="s">
+        <v>454</v>
+      </c>
+      <c r="F1" s="43" t="s">
+        <v>455</v>
+      </c>
+      <c r="G1" s="43" t="s">
+        <v>456</v>
+      </c>
+      <c r="H1" s="43" t="s">
+        <v>457</v>
+      </c>
+      <c r="I1" s="43" t="s">
+        <v>458</v>
+      </c>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="42"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -13615,13 +13595,13 @@
         <v>404</v>
       </c>
       <c r="R1" s="47" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="S1" s="47" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="T1" s="47" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="U1" s="8"/>
       <c r="V1" s="8"/>

</xml_diff>